<commit_message>
Dependency map: count rework that iteration loops trigger in the to-do list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/06-wrapup/CFU-000-PM-DEP-001_Design-Dependency-Map.xlsx
+++ b/deliverables/06-wrapup/CFU-000-PM-DEP-001_Design-Dependency-Map.xlsx
@@ -10782,7 +10782,11 @@
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>PRC-02, PRC-03, PRC-04, LAY-01, ELE-01, PRC-06, PRC-07, MEC-01, LAY-02, ICS-01, ELE-02, ELE-03, PRC-08, MEC-02, MEC-03, ELE-04, CST-01, SAF-01, PIP-02, ICS-04, ICS-05, PIP-03, PIP-04, ICS-02, ICS-06, ICS-07, ICS-03, PRJ-03</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Governing case (C-101 reflux failure, about 220 t/h) needs power and cooling-water failure cases.</t>
@@ -10814,7 +10818,11 @@
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>PRC-02, PRC-03, PRC-04, LAY-01, ELE-01, PRC-06, PRC-07, MEC-01, LAY-02, ICS-01, ELE-02, ELE-03, PRC-08, MEC-02, MEC-03, ELE-04, CST-01, SAF-01, PIP-02, ICS-04, ICS-05, PIP-03, PIP-04, ICS-02, ICS-06, ICS-07, ICS-03, PRJ-03</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Vendor data revises weights, nozzles, motor ratings and I/O; plan for one full update cycle.</t>
@@ -10846,7 +10854,11 @@
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>PRC-02, PRC-03, PRC-04, LAY-01, ELE-01, PRC-06, PRC-07, MEC-01, LAY-02, ICS-01, ELE-02, ELE-03, PRC-08, MEC-02, MEC-03, ELE-04, CST-01, SAF-01, PIP-02, ICS-04, ICS-05, PIP-03, PIP-04, ICS-02, ICS-06, ICS-07, ICS-03, PRJ-03</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>API 752/753 siting, QRA, fire and gas mapping and fireproofing; may move buildings or equipment.</t>
@@ -10986,7 +10998,11 @@
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>PRC-02, PRC-03, PRC-04, LAY-01, ELE-01, PRC-06, PRC-07, MEC-01, LAY-02, ICS-01, ELE-02, ELE-03, PRC-08, MEC-02, MEC-03, ELE-04, CST-01, SAF-01, PIP-02, ICS-04, ICS-05, PIP-03, PIP-04, ICS-02, ICS-06, ICS-07, ICS-03, PRJ-03</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Phase maturity plan: carry the dependency map through FEL 1-3 and detailed design
Adds a maturity scale, gate targets for every activity, 16 phase-only activities
(business case, select decision, execution plan, procurement, work packaging,
detail design) and the maturity each link needs. Iteration loops become forward
links between levels, so the step network has no cycles. The build checks gate
consistency and compares targets with what the package has issued.

New outputs: CFU-000-PM-DEP-003 report and workbook, portal/phases.html.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/06-wrapup/CFU-000-PM-DEP-001_Design-Dependency-Map.xlsx
+++ b/deliverables/06-wrapup/CFU-000-PM-DEP-001_Design-Dependency-Map.xlsx
@@ -563,7 +563,7 @@
         <v>44</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         <v>43</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         <v>42</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         <v>41</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
     </row>
@@ -782,7 +782,7 @@
         <v>38</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
         <v>2</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7" s="2" t="inlineStr"/>
     </row>
@@ -885,7 +885,7 @@
         <v>20</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>28</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
     </row>
@@ -989,7 +989,7 @@
         <v>24</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M10" s="2" t="inlineStr"/>
     </row>
@@ -1044,7 +1044,7 @@
         <v>23</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M11" s="2" t="inlineStr"/>
     </row>
@@ -1093,7 +1093,7 @@
         <v>7</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M12" s="2" t="inlineStr"/>
     </row>
@@ -1144,7 +1144,7 @@
         <v>20</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M13" s="2" t="inlineStr"/>
     </row>
@@ -1195,7 +1195,7 @@
         <v>2</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M14" s="2" t="inlineStr"/>
     </row>
@@ -1303,7 +1303,7 @@
         <v>15</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M16" s="2" t="inlineStr"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>3</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M17" s="2" t="inlineStr"/>
     </row>
@@ -1404,7 +1404,7 @@
         <v>2</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M18" s="2" t="inlineStr"/>
     </row>
@@ -1455,7 +1455,7 @@
         <v>5</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M19" s="2" t="inlineStr"/>
     </row>
@@ -1508,7 +1508,7 @@
         <v>6</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M20" s="2" t="inlineStr"/>
     </row>
@@ -1566,7 +1566,7 @@
         <v>19</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         <v>7</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M22" s="2" t="inlineStr"/>
     </row>
@@ -1670,7 +1670,7 @@
         <v>2</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M23" s="2" t="inlineStr"/>
     </row>
@@ -1722,7 +1722,7 @@
         <v>3</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M24" s="2" t="inlineStr"/>
     </row>
@@ -1772,7 +1772,7 @@
         <v>3</v>
       </c>
       <c r="L25" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M25" s="2" t="inlineStr"/>
     </row>
@@ -1823,7 +1823,7 @@
         <v>7</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M26" s="2" t="inlineStr"/>
     </row>
@@ -1932,7 +1932,7 @@
         <v>8</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M28" s="2" t="inlineStr"/>
     </row>
@@ -1984,7 +1984,7 @@
         <v>2</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M29" s="2" t="inlineStr"/>
     </row>
@@ -2040,7 +2040,7 @@
         <v>4</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M30" s="2" t="inlineStr"/>
     </row>
@@ -2145,7 +2145,7 @@
         <v>6</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
@@ -2199,7 +2199,7 @@
         <v>3</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M33" s="2" t="inlineStr"/>
     </row>
@@ -2249,7 +2249,7 @@
         <v>5</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
@@ -2302,7 +2302,7 @@
         <v>2</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M35" s="2" t="inlineStr"/>
     </row>
@@ -2352,7 +2352,7 @@
         <v>2</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M36" s="2" t="inlineStr"/>
     </row>
@@ -2620,7 +2620,7 @@
         <v>2</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M41" s="2" t="inlineStr"/>
     </row>
@@ -2671,7 +2671,7 @@
       <c r="H42" s="2" t="inlineStr"/>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-ME-LST-001, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PI-SPC-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-BFD-001, CFU-000-PR-BOD-001, CFU-000-PR-HMB-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-ME-LST-001, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PI-SPC-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-BFD-001, CFU-000-PR-BOD-001, CFU-000-PR-HMB-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9681,7 +9681,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-ME-LST-001, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PI-SPC-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-BFD-001, CFU-000-PR-HMB-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-ME-LST-001, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PI-SPC-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-BFD-001, CFU-000-PR-HMB-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9703,7 +9703,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-ME-LST-001, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PI-SPC-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-BFD-001, CFU-000-PR-HMB-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-ME-LST-001, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PI-SPC-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-BFD-001, CFU-000-PR-HMB-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-ME-LST-001, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PI-SPC-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-BFD-001, CFU-000-PR-HMB-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-ME-LST-001, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PI-SPC-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-BFD-001, CFU-000-PR-HMB-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9747,7 +9747,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-ME-LST-001, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-ME-LST-001, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9769,7 +9769,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-002, CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-001, CFU-000-PR-RPT-002, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9791,7 +9791,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-001, CFU-000-IC-RPT-002, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-002, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-IC-CSD-005, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9813,7 +9813,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-002, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-002, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-PI-ISO-001, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-002, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PL-PLT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-002, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-PI-ISO-001, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-002, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-002, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-002, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-000-PR-PFD-ALL, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-002, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PFD-001, CFU-100-PR-PFD-002, CFU-100-PR-PFD-003, CFU-100-PR-PFD-004, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-PI-ISO-001, CFU-200-PR-PFD-005, CFU-200-PR-PFD-006, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9857,7 +9857,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-002, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PI-SPC-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-002, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-PI-ISO-001, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-002, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PI-SPC-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-002, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-PI-ISO-001, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-002, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-002, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-PI-ISO-001, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
+          <t>CFU-000-IC-BLK-001, CFU-000-IC-CAL-001, CFU-000-IC-CE-001, CFU-000-IC-IDX-001, CFU-000-IC-IOL-001, CFU-000-IC-RPT-002, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-LL-001, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-000-PR-PID-000, CFU-000-PR-PID-ALL, CFU-000-PR-RPT-002, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-100-PR-PID-001, CFU-100-PR-PID-002, CFU-100-PR-PID-003, CFU-100-PR-PID-004, CFU-100-PR-PID-005, CFU-100-PR-PID-006, CFU-100-PR-PID-007, CFU-100-PR-PID-008, CFU-100-PR-PID-009, CFU-100-PR-PID-010, CFU-100-PR-PID-011, CFU-200-PI-ISO-001, CFU-200-PR-PID-012, CFU-200-PR-PID-013, CFU-200-PR-PID-014, CFU-200-PR-PID-015, CFU-900-PR-PID-016</t>
         </is>
       </c>
     </row>
@@ -9901,7 +9901,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001</t>
+          <t>CFU-000-ME-CAL-001, CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-EST-001, CFU-000-PM-REG-001, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-200-ME-GA-004, CFU-200-ME-GA-006, CFU-200-PI-ISO-001</t>
         </is>
       </c>
     </row>
@@ -9923,7 +9923,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-200-PI-ISO-001</t>
+          <t>CFU-000-PI-3DM-002, CFU-000-PI-ISO-000, CFU-000-PI-MTO-001, CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-200-PI-ISO-001</t>
         </is>
       </c>
     </row>
@@ -9945,7 +9945,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-CE-001, CFU-000-IC-RPT-002, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-000-PR-RPT-002</t>
+          <t>CFU-000-IC-CE-001, CFU-000-IC-RPT-002, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-000-PR-RPT-002</t>
         </is>
       </c>
     </row>
@@ -9967,7 +9967,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-ME-DS-000, CFU-000-ME-DS-001, CFU-000-ME-DS-002, CFU-000-ME-DS-003, CFU-000-ME-DS-004, CFU-000-ME-DS-005, CFU-000-ME-DS-006, CFU-000-ME-DS-007, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -9989,7 +9989,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-LDL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10011,7 +10011,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-PI-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10033,7 +10033,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-EL-CAL-001, CFU-000-EL-CBL-001, CFU-000-EL-SLD-001, CFU-000-EL-SLD-002, CFU-000-EL-SLD-003, CFU-000-EL-SLD-004, CFU-000-IC-BLK-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10073,7 +10073,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-CE-001, CFU-000-IC-RPT-002, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-IC-CE-001, CFU-000-IC-RPT-002, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10095,7 +10095,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-EL-CBL-001, CFU-000-EL-HAC-001, CFU-000-EL-HAC-002, CFU-000-EL-HAC-003, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10117,7 +10117,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-BLK-001, CFU-000-IC-IOL-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL</t>
+          <t>CFU-000-IC-BLK-001, CFU-000-IC-IOL-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL</t>
         </is>
       </c>
     </row>
@@ -10139,7 +10139,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-PL-3DM-001, CFU-000-PL-ELV-001, CFU-000-PL-ELV-002, CFU-000-PL-ELV-003, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10161,7 +10161,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PI-ISO-000, CFU-000-PI-MTO-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-200-PI-ISO-001</t>
+          <t>CFU-000-PI-ISO-000, CFU-000-PI-MTO-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-100-PI-ISO-001, CFU-100-PI-ISO-002, CFU-100-PI-ISO-003, CFU-100-PI-ISO-004, CFU-100-PI-ISO-005, CFU-100-PI-ISO-006, CFU-100-PI-ISO-007, CFU-100-PI-ISO-008, CFU-100-PI-ISO-009, CFU-100-PI-ISO-010, CFU-100-PI-ISO-011, CFU-100-PI-ISO-012, CFU-200-PI-ISO-001</t>
         </is>
       </c>
     </row>
@@ -10201,7 +10201,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-EL-CBL-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-EL-CBL-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10223,7 +10223,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-EST-001, CFU-000-PM-REG-001</t>
+          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-EST-001, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10245,7 +10245,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-000-PR-BFD-001</t>
+          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-000-PR-BFD-001</t>
         </is>
       </c>
     </row>
@@ -10267,7 +10267,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-000-PR-RPT-001</t>
+          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-000-PR-RPT-001</t>
         </is>
       </c>
     </row>
@@ -10307,7 +10307,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-200-ME-GA-004, CFU-200-ME-GA-006</t>
+          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-100-ME-GA-001, CFU-100-ME-GA-002, CFU-100-ME-GA-003, CFU-100-ME-GA-005, CFU-100-ME-GA-007, CFU-100-ME-GA-008, CFU-200-ME-GA-004, CFU-200-ME-GA-006</t>
         </is>
       </c>
     </row>
@@ -10329,7 +10329,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-200-IC-CSD-005</t>
+          <t>CFU-000-IC-CSD-006, CFU-000-IC-CSD-ALL, CFU-000-IC-RPT-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-100-IC-CSD-001, CFU-100-IC-CSD-002, CFU-100-IC-CSD-003, CFU-100-IC-CSD-004, CFU-200-IC-CSD-005</t>
         </is>
       </c>
     </row>
@@ -10351,7 +10351,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-CE-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-IC-CE-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10373,7 +10373,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-CAL-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-IC-CAL-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10395,7 +10395,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL</t>
+          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001, CFU-100-IC-LD-001, CFU-100-IC-LD-002, CFU-100-IC-LD-003, CFU-100-IC-LD-ALL</t>
         </is>
       </c>
     </row>
@@ -10417,7 +10417,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-IC-BLK-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-IC-BLK-001, CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>
@@ -10565,7 +10565,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-REG-001</t>
+          <t>CFU-000-PM-DEP-001, CFU-000-PM-DEP-002, CFU-000-PM-DEP-003, CFU-000-PM-REG-001</t>
         </is>
       </c>
     </row>

</xml_diff>